<commit_message>
Updatedes shematics only to REV 2 which only shows changes necessary to make work. Final edits of UMTS. Updated audio files. Repo Clean up.
</commit_message>
<xml_diff>
--- a/Hardware/Softcore_SA_HW/Default Configuration/Outputs/BOM/BOM_PartType-Softcore_SA_HW.xlsx
+++ b/Hardware/Softcore_SA_HW/Default Configuration/Outputs/BOM/BOM_PartType-Softcore_SA_HW.xlsx
@@ -1,14 +1,9 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\IMR_Projects\IMR\Softcore_SA\Hardware\Softcore_SA_HW\Default Configuration\Outputs\BOM\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{613BD6A7-BA99-4805-B2F1-8BF393435C70}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{9420F368-470C-491B-A118-1198F08037D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -132,10 +127,10 @@
     <t>None</t>
   </si>
   <si>
-    <t>1/25/2026</t>
-  </si>
-  <si>
-    <t>8:30:27 AM</t>
+    <t>3/22/2026</t>
+  </si>
+  <si>
+    <t>6:07:15 PM</t>
   </si>
   <si>
     <t>SoftCore SA Adapter</t>
@@ -144,7 +139,7 @@
     <t>IMR-006-SCH</t>
   </si>
   <si>
-    <t>1</t>
+    <t>2</t>
   </si>
   <si>
     <t>Hab S Collector</t>
@@ -1404,7 +1399,7 @@
     <t>192</t>
   </si>
   <si>
-    <t>1/25/2026 8:30:27 AM</t>
+    <t>3/22/2026 6:07:15 PM</t>
   </si>
   <si>
     <t>BOM_PartType</t>
@@ -2146,51 +2141,6 @@
     <xf numFmtId="166" fontId="7" fillId="7" borderId="22" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="29" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="6" borderId="31" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="166" fontId="7" fillId="5" borderId="32" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
@@ -2198,6 +2148,51 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="left" vertical="top"/>
       <protection locked="0"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="4" borderId="2" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="2" borderId="7" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="29" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="11" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="26" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="27" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="6" borderId="31" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="166" fontId="7" fillId="5" borderId="32" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="17" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="5" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2292,15 +2287,15 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>8</xdr:col>
-      <xdr:colOff>733425</xdr:colOff>
+      <xdr:colOff>304800</xdr:colOff>
       <xdr:row>2</xdr:row>
-      <xdr:rowOff>28575</xdr:rowOff>
+      <xdr:rowOff>76200</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>11</xdr:col>
-      <xdr:colOff>85725</xdr:colOff>
+      <xdr:colOff>619125</xdr:colOff>
       <xdr:row>7</xdr:row>
-      <xdr:rowOff>92869</xdr:rowOff>
+      <xdr:rowOff>95250</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -2328,8 +2323,8 @@
       </xdr:blipFill>
       <xdr:spPr bwMode="auto">
         <a:xfrm>
-          <a:off x="12077700" y="657225"/>
-          <a:ext cx="3495675" cy="873919"/>
+          <a:off x="11649075" y="723900"/>
+          <a:ext cx="4457700" cy="1114425"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -2655,7 +2650,7 @@
       <c r="L1" s="18"/>
       <c r="M1" s="22"/>
     </row>
-    <row r="2" spans="1:13" ht="36" thickBot="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:13" ht="37.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A2" s="14"/>
       <c r="B2" s="40"/>
       <c r="C2" s="40"/>
@@ -2664,7 +2659,7 @@
       </c>
       <c r="E2" s="40"/>
       <c r="F2" s="41"/>
-      <c r="G2" s="62" t="s">
+      <c r="G2" s="64" t="s">
         <v>35</v>
       </c>
       <c r="H2" s="23"/>
@@ -2673,21 +2668,21 @@
       <c r="K2" s="23"/>
       <c r="L2" s="24"/>
     </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:13" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A3" s="14"/>
       <c r="B3" s="26"/>
       <c r="C3" s="26"/>
       <c r="D3" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="E3" s="58" t="s">
+      <c r="E3" s="60" t="s">
         <v>31</v>
       </c>
       <c r="F3" s="27"/>
       <c r="G3" s="28" t="s">
         <v>25</v>
       </c>
-      <c r="H3" s="58" t="s">
+      <c r="H3" s="60" t="s">
         <v>36</v>
       </c>
       <c r="I3" s="26"/>
@@ -2695,21 +2690,21 @@
       <c r="K3" s="26"/>
       <c r="L3" s="30"/>
     </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A4" s="14"/>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
       <c r="D4" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="E4" s="59" t="s">
+      <c r="E4" s="61" t="s">
         <v>31</v>
       </c>
       <c r="F4" s="27"/>
       <c r="G4" s="31" t="s">
         <v>26</v>
       </c>
-      <c r="H4" s="59" t="s">
+      <c r="H4" s="61" t="s">
         <v>37</v>
       </c>
       <c r="I4" s="29"/>
@@ -2717,21 +2712,21 @@
       <c r="K4" s="29"/>
       <c r="L4" s="30"/>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:13" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="14"/>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="E5" s="60" t="s">
+      <c r="E5" s="62" t="s">
         <v>32</v>
       </c>
       <c r="F5" s="27"/>
       <c r="G5" s="32" t="s">
         <v>27</v>
       </c>
-      <c r="H5" s="60" t="s">
+      <c r="H5" s="62" t="s">
         <v>38</v>
       </c>
       <c r="I5" s="29"/>
@@ -2753,17 +2748,17 @@
       <c r="K6" s="29"/>
       <c r="L6" s="36"/>
     </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="14"/>
       <c r="B7" s="37"/>
       <c r="C7" s="37"/>
       <c r="D7" s="29" t="s">
         <v>18</v>
       </c>
-      <c r="E7" s="61" t="s">
+      <c r="E7" s="63" t="s">
         <v>33</v>
       </c>
-      <c r="F7" s="61" t="s">
+      <c r="F7" s="63" t="s">
         <v>34</v>
       </c>
       <c r="H7" s="37"/>
@@ -2772,7 +2767,7 @@
       <c r="K7" s="37"/>
       <c r="L7" s="30"/>
     </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:13" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="14"/>
       <c r="B8" s="33"/>
       <c r="C8" s="33"/>
@@ -2781,11 +2776,11 @@
       </c>
       <c r="E8" s="38">
         <f ca="1">TODAY()</f>
-        <v>46047</v>
+        <v>46103</v>
       </c>
       <c r="F8" s="39">
         <f ca="1">NOW()</f>
-        <v>46047.3570400463</v>
+        <v>46103.755445023147</v>
       </c>
       <c r="H8" s="37"/>
       <c r="I8" s="37"/>
@@ -2793,36 +2788,36 @@
       <c r="K8" s="37"/>
       <c r="L8" s="30"/>
     </row>
-    <row r="9" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:13" s="2" customFormat="1" ht="18" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A9" s="14"/>
       <c r="B9" s="45" t="s">
         <v>21</v>
       </c>
-      <c r="C9" s="63" t="s">
+      <c r="C9" s="65" t="s">
         <v>39</v>
       </c>
-      <c r="D9" s="64" t="s">
+      <c r="D9" s="66" t="s">
         <v>40</v>
       </c>
-      <c r="E9" s="64" t="s">
+      <c r="E9" s="66" t="s">
         <v>109</v>
       </c>
-      <c r="F9" s="64" t="s">
+      <c r="F9" s="66" t="s">
         <v>174</v>
       </c>
-      <c r="G9" s="64" t="s">
+      <c r="G9" s="66" t="s">
         <v>243</v>
       </c>
-      <c r="H9" s="64" t="s">
+      <c r="H9" s="66" t="s">
         <v>273</v>
       </c>
-      <c r="I9" s="64" t="s">
+      <c r="I9" s="66" t="s">
         <v>342</v>
       </c>
-      <c r="J9" s="64" t="s">
+      <c r="J9" s="66" t="s">
         <v>346</v>
       </c>
-      <c r="K9" s="64" t="s">
+      <c r="K9" s="66" t="s">
         <v>413</v>
       </c>
       <c r="L9" s="25" t="s">
@@ -2832,34 +2827,34 @@
     <row r="10" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="14"/>
       <c r="B10" s="48">
-        <f t="shared" ref="B10:B41" si="0">ROW(B10) - ROW($B$9)</f>
+        <f>ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
       <c r="C10" s="50">
         <v>5</v>
       </c>
-      <c r="D10" s="65" t="s">
+      <c r="D10" s="67" t="s">
         <v>41</v>
       </c>
-      <c r="E10" s="65" t="s">
+      <c r="E10" s="67" t="s">
         <v>110</v>
       </c>
-      <c r="F10" s="67" t="s">
+      <c r="F10" s="69" t="s">
         <v>175</v>
       </c>
-      <c r="G10" s="67" t="s">
+      <c r="G10" s="69" t="s">
         <v>244</v>
       </c>
-      <c r="H10" s="67" t="s">
+      <c r="H10" s="69" t="s">
         <v>274</v>
       </c>
-      <c r="I10" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J10" s="67" t="s">
+      <c r="I10" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J10" s="69" t="s">
         <v>347</v>
       </c>
-      <c r="K10" s="68" t="s">
+      <c r="K10" s="70" t="s">
         <v>414</v>
       </c>
       <c r="L10" s="55">
@@ -2867,75 +2862,75 @@
         <v>1.4000000000000001</v>
       </c>
     </row>
-    <row r="11" spans="1:13" s="3" customFormat="1" ht="33.75" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:13" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A11" s="14"/>
       <c r="B11" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B11) - ROW($B$9)</f>
         <v>2</v>
       </c>
       <c r="C11" s="51">
         <v>18</v>
       </c>
-      <c r="D11" s="66" t="s">
+      <c r="D11" s="68" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="66" t="s">
+      <c r="E11" s="68" t="s">
         <v>111</v>
       </c>
-      <c r="F11" s="66" t="s">
+      <c r="F11" s="68" t="s">
         <v>176</v>
       </c>
-      <c r="G11" s="66" t="s">
+      <c r="G11" s="68" t="s">
         <v>245</v>
       </c>
-      <c r="H11" s="66" t="s">
+      <c r="H11" s="68" t="s">
         <v>275</v>
       </c>
-      <c r="I11" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J11" s="66" t="s">
+      <c r="I11" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J11" s="68" t="s">
         <v>348</v>
       </c>
-      <c r="K11" s="69" t="s">
+      <c r="K11" s="71" t="s">
         <v>415</v>
       </c>
       <c r="L11" s="57">
-        <f t="shared" ref="L11" si="1">C11*K11</f>
+        <f t="shared" ref="L11:L77" si="0">C11*K11</f>
         <v>1.8</v>
       </c>
     </row>
     <row r="12" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="14"/>
       <c r="B12" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B12) - ROW($B$9)</f>
         <v>3</v>
       </c>
       <c r="C12" s="50">
         <v>1</v>
       </c>
-      <c r="D12" s="65" t="s">
+      <c r="D12" s="67" t="s">
         <v>43</v>
       </c>
-      <c r="E12" s="65" t="s">
+      <c r="E12" s="67" t="s">
         <v>112</v>
       </c>
-      <c r="F12" s="67" t="s">
+      <c r="F12" s="69" t="s">
         <v>177</v>
       </c>
-      <c r="G12" s="67" t="s">
+      <c r="G12" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H12" s="67" t="s">
+      <c r="H12" s="69" t="s">
         <v>276</v>
       </c>
-      <c r="I12" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J12" s="67" t="s">
+      <c r="I12" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J12" s="69" t="s">
         <v>349</v>
       </c>
-      <c r="K12" s="68" t="s">
+      <c r="K12" s="70" t="s">
         <v>416</v>
       </c>
       <c r="L12" s="55">
@@ -2943,75 +2938,75 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="13" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:13" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A13" s="14"/>
       <c r="B13" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B13) - ROW($B$9)</f>
         <v>4</v>
       </c>
       <c r="C13" s="51">
         <v>5</v>
       </c>
-      <c r="D13" s="66" t="s">
+      <c r="D13" s="68" t="s">
         <v>44</v>
       </c>
-      <c r="E13" s="66" t="s">
+      <c r="E13" s="68" t="s">
         <v>113</v>
       </c>
-      <c r="F13" s="66" t="s">
+      <c r="F13" s="68" t="s">
         <v>178</v>
       </c>
-      <c r="G13" s="66" t="s">
+      <c r="G13" s="68" t="s">
         <v>244</v>
       </c>
-      <c r="H13" s="66" t="s">
+      <c r="H13" s="68" t="s">
         <v>277</v>
       </c>
-      <c r="I13" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J13" s="66" t="s">
+      <c r="I13" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J13" s="68" t="s">
         <v>350</v>
       </c>
-      <c r="K13" s="69" t="s">
+      <c r="K13" s="71" t="s">
         <v>414</v>
       </c>
       <c r="L13" s="57">
-        <f t="shared" ref="L13" si="2">C13*K13</f>
+        <f t="shared" ref="L13" si="1">C13*K13</f>
         <v>1.4000000000000001</v>
       </c>
     </row>
     <row r="14" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="14"/>
       <c r="B14" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B14) - ROW($B$9)</f>
         <v>5</v>
       </c>
       <c r="C14" s="50">
         <v>2</v>
       </c>
-      <c r="D14" s="65" t="s">
+      <c r="D14" s="67" t="s">
         <v>45</v>
       </c>
-      <c r="E14" s="65" t="s">
+      <c r="E14" s="67" t="s">
         <v>114</v>
       </c>
-      <c r="F14" s="67" t="s">
+      <c r="F14" s="69" t="s">
         <v>179</v>
       </c>
-      <c r="G14" s="67" t="s">
+      <c r="G14" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H14" s="67" t="s">
+      <c r="H14" s="69" t="s">
         <v>278</v>
       </c>
-      <c r="I14" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J14" s="67" t="s">
+      <c r="I14" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J14" s="69" t="s">
         <v>351</v>
       </c>
-      <c r="K14" s="68" t="s">
+      <c r="K14" s="70" t="s">
         <v>416</v>
       </c>
       <c r="L14" s="55">
@@ -3019,75 +3014,75 @@
         <v>0.22</v>
       </c>
     </row>
-    <row r="15" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:13" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A15" s="14"/>
       <c r="B15" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B15) - ROW($B$9)</f>
         <v>6</v>
       </c>
       <c r="C15" s="51">
         <v>2</v>
       </c>
-      <c r="D15" s="66" t="s">
+      <c r="D15" s="68" t="s">
         <v>46</v>
       </c>
-      <c r="E15" s="66" t="s">
+      <c r="E15" s="68" t="s">
         <v>115</v>
       </c>
-      <c r="F15" s="66" t="s">
+      <c r="F15" s="68" t="s">
         <v>180</v>
       </c>
-      <c r="G15" s="66" t="s">
+      <c r="G15" s="68" t="s">
         <v>244</v>
       </c>
-      <c r="H15" s="66" t="s">
+      <c r="H15" s="68" t="s">
         <v>279</v>
       </c>
-      <c r="I15" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J15" s="66" t="s">
+      <c r="I15" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J15" s="68" t="s">
         <v>352</v>
       </c>
-      <c r="K15" s="69" t="s">
+      <c r="K15" s="71" t="s">
         <v>417</v>
       </c>
       <c r="L15" s="57">
-        <f t="shared" ref="L15" si="3">C15*K15</f>
+        <f t="shared" ref="L15" si="2">C15*K15</f>
         <v>0.26</v>
       </c>
     </row>
     <row r="16" spans="1:13" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="14"/>
       <c r="B16" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B16) - ROW($B$9)</f>
         <v>7</v>
       </c>
       <c r="C16" s="50">
         <v>2</v>
       </c>
-      <c r="D16" s="65" t="s">
+      <c r="D16" s="67" t="s">
         <v>47</v>
       </c>
-      <c r="E16" s="65" t="s">
+      <c r="E16" s="67" t="s">
         <v>116</v>
       </c>
-      <c r="F16" s="67" t="s">
+      <c r="F16" s="69" t="s">
         <v>181</v>
       </c>
-      <c r="G16" s="67" t="s">
+      <c r="G16" s="69" t="s">
         <v>245</v>
       </c>
-      <c r="H16" s="67" t="s">
+      <c r="H16" s="69" t="s">
         <v>280</v>
       </c>
-      <c r="I16" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J16" s="67" t="s">
+      <c r="I16" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J16" s="69" t="s">
         <v>353</v>
       </c>
-      <c r="K16" s="68" t="s">
+      <c r="K16" s="70" t="s">
         <v>418</v>
       </c>
       <c r="L16" s="55">
@@ -3095,75 +3090,75 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="17" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="14"/>
       <c r="B17" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B17) - ROW($B$9)</f>
         <v>8</v>
       </c>
       <c r="C17" s="51">
         <v>2</v>
       </c>
-      <c r="D17" s="66" t="s">
+      <c r="D17" s="68" t="s">
         <v>48</v>
       </c>
-      <c r="E17" s="66" t="s">
+      <c r="E17" s="68" t="s">
         <v>117</v>
       </c>
-      <c r="F17" s="66" t="s">
+      <c r="F17" s="68" t="s">
         <v>182</v>
       </c>
-      <c r="G17" s="66" t="s">
+      <c r="G17" s="68" t="s">
         <v>247</v>
       </c>
-      <c r="H17" s="66" t="s">
+      <c r="H17" s="68" t="s">
         <v>281</v>
       </c>
-      <c r="I17" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J17" s="66" t="s">
+      <c r="I17" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J17" s="68" t="s">
         <v>354</v>
       </c>
-      <c r="K17" s="69" t="s">
+      <c r="K17" s="71" t="s">
         <v>419</v>
       </c>
       <c r="L17" s="57">
-        <f t="shared" ref="L17" si="4">C17*K17</f>
+        <f t="shared" ref="L17" si="3">C17*K17</f>
         <v>0.24</v>
       </c>
     </row>
     <row r="18" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="14"/>
       <c r="B18" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B18) - ROW($B$9)</f>
         <v>9</v>
       </c>
       <c r="C18" s="50">
         <v>3</v>
       </c>
-      <c r="D18" s="65" t="s">
+      <c r="D18" s="67" t="s">
         <v>49</v>
       </c>
-      <c r="E18" s="65" t="s">
+      <c r="E18" s="67" t="s">
         <v>118</v>
       </c>
-      <c r="F18" s="67" t="s">
+      <c r="F18" s="69" t="s">
         <v>183</v>
       </c>
-      <c r="G18" s="67" t="s">
+      <c r="G18" s="69" t="s">
         <v>248</v>
       </c>
-      <c r="H18" s="67" t="s">
+      <c r="H18" s="69" t="s">
         <v>282</v>
       </c>
-      <c r="I18" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J18" s="67" t="s">
+      <c r="I18" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J18" s="69" t="s">
         <v>355</v>
       </c>
-      <c r="K18" s="68" t="s">
+      <c r="K18" s="70" t="s">
         <v>420</v>
       </c>
       <c r="L18" s="55">
@@ -3171,75 +3166,75 @@
         <v>5.76</v>
       </c>
     </row>
-    <row r="19" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="14"/>
       <c r="B19" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B19) - ROW($B$9)</f>
         <v>10</v>
       </c>
       <c r="C19" s="51">
         <v>3</v>
       </c>
-      <c r="D19" s="66" t="s">
+      <c r="D19" s="68" t="s">
         <v>50</v>
       </c>
-      <c r="E19" s="66" t="s">
+      <c r="E19" s="68" t="s">
         <v>119</v>
       </c>
-      <c r="F19" s="66" t="s">
+      <c r="F19" s="68" t="s">
         <v>184</v>
       </c>
-      <c r="G19" s="66" t="s">
+      <c r="G19" s="68" t="s">
         <v>244</v>
       </c>
-      <c r="H19" s="66" t="s">
+      <c r="H19" s="68" t="s">
         <v>283</v>
       </c>
-      <c r="I19" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J19" s="66" t="s">
+      <c r="I19" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J19" s="68" t="s">
         <v>356</v>
       </c>
-      <c r="K19" s="69" t="s">
+      <c r="K19" s="71" t="s">
         <v>421</v>
       </c>
       <c r="L19" s="57">
-        <f t="shared" ref="L19" si="5">C19*K19</f>
+        <f t="shared" ref="L19" si="4">C19*K19</f>
         <v>0.57000000000000006</v>
       </c>
     </row>
     <row r="20" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="14"/>
       <c r="B20" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B20) - ROW($B$9)</f>
         <v>11</v>
       </c>
       <c r="C20" s="50">
         <v>1</v>
       </c>
-      <c r="D20" s="65" t="s">
+      <c r="D20" s="67" t="s">
         <v>51</v>
       </c>
-      <c r="E20" s="65" t="s">
+      <c r="E20" s="67" t="s">
         <v>120</v>
       </c>
-      <c r="F20" s="67" t="s">
+      <c r="F20" s="69" t="s">
         <v>185</v>
       </c>
-      <c r="G20" s="67" t="s">
+      <c r="G20" s="69" t="s">
         <v>247</v>
       </c>
-      <c r="H20" s="67" t="s">
+      <c r="H20" s="69" t="s">
         <v>284</v>
       </c>
-      <c r="I20" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J20" s="67" t="s">
+      <c r="I20" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J20" s="69" t="s">
         <v>357</v>
       </c>
-      <c r="K20" s="68" t="s">
+      <c r="K20" s="70" t="s">
         <v>422</v>
       </c>
       <c r="L20" s="55">
@@ -3247,75 +3242,75 @@
         <v>0.24</v>
       </c>
     </row>
-    <row r="21" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="14"/>
       <c r="B21" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B21) - ROW($B$9)</f>
         <v>12</v>
       </c>
       <c r="C21" s="51">
         <v>1</v>
       </c>
-      <c r="D21" s="66" t="s">
+      <c r="D21" s="68" t="s">
         <v>52</v>
       </c>
-      <c r="E21" s="66" t="s">
+      <c r="E21" s="68" t="s">
         <v>121</v>
       </c>
-      <c r="F21" s="66" t="s">
+      <c r="F21" s="68" t="s">
         <v>186</v>
       </c>
-      <c r="G21" s="66" t="s">
+      <c r="G21" s="68" t="s">
         <v>244</v>
       </c>
-      <c r="H21" s="66" t="s">
+      <c r="H21" s="68" t="s">
         <v>285</v>
       </c>
-      <c r="I21" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J21" s="66" t="s">
+      <c r="I21" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J21" s="68" t="s">
         <v>358</v>
       </c>
-      <c r="K21" s="69" t="s">
+      <c r="K21" s="71" t="s">
         <v>423</v>
       </c>
       <c r="L21" s="57">
-        <f t="shared" ref="L21" si="6">C21*K21</f>
+        <f t="shared" ref="L21" si="5">C21*K21</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="22" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="14"/>
       <c r="B22" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B22) - ROW($B$9)</f>
         <v>13</v>
       </c>
       <c r="C22" s="50">
         <v>1</v>
       </c>
-      <c r="D22" s="65" t="s">
+      <c r="D22" s="67" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="65" t="s">
+      <c r="E22" s="67" t="s">
         <v>122</v>
       </c>
-      <c r="F22" s="67" t="s">
+      <c r="F22" s="69" t="s">
         <v>187</v>
       </c>
-      <c r="G22" s="67" t="s">
+      <c r="G22" s="69" t="s">
         <v>247</v>
       </c>
-      <c r="H22" s="67" t="s">
+      <c r="H22" s="69" t="s">
         <v>286</v>
       </c>
-      <c r="I22" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J22" s="67" t="s">
+      <c r="I22" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J22" s="69" t="s">
         <v>359</v>
       </c>
-      <c r="K22" s="68" t="s">
+      <c r="K22" s="70" t="s">
         <v>416</v>
       </c>
       <c r="L22" s="55">
@@ -3323,75 +3318,75 @@
         <v>0.11</v>
       </c>
     </row>
-    <row r="23" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="14"/>
       <c r="B23" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B23) - ROW($B$9)</f>
         <v>14</v>
       </c>
       <c r="C23" s="51">
         <v>1</v>
       </c>
-      <c r="D23" s="66" t="s">
+      <c r="D23" s="68" t="s">
         <v>54</v>
       </c>
-      <c r="E23" s="66" t="s">
+      <c r="E23" s="68" t="s">
         <v>123</v>
       </c>
-      <c r="F23" s="66" t="s">
+      <c r="F23" s="68" t="s">
         <v>188</v>
       </c>
-      <c r="G23" s="66" t="s">
+      <c r="G23" s="68" t="s">
         <v>244</v>
       </c>
-      <c r="H23" s="66" t="s">
+      <c r="H23" s="68" t="s">
         <v>287</v>
       </c>
-      <c r="I23" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J23" s="66" t="s">
+      <c r="I23" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J23" s="68" t="s">
         <v>360</v>
       </c>
-      <c r="K23" s="69" t="s">
+      <c r="K23" s="71" t="s">
         <v>424</v>
       </c>
       <c r="L23" s="57">
-        <f t="shared" ref="L23" si="7">C23*K23</f>
+        <f t="shared" ref="L23" si="6">C23*K23</f>
         <v>0.38</v>
       </c>
     </row>
     <row r="24" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="14"/>
       <c r="B24" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B24) - ROW($B$9)</f>
         <v>15</v>
       </c>
       <c r="C24" s="50">
         <v>8</v>
       </c>
-      <c r="D24" s="65" t="s">
+      <c r="D24" s="67" t="s">
         <v>55</v>
       </c>
-      <c r="E24" s="65" t="s">
+      <c r="E24" s="67" t="s">
         <v>124</v>
       </c>
-      <c r="F24" s="67" t="s">
+      <c r="F24" s="69" t="s">
         <v>189</v>
       </c>
-      <c r="G24" s="67" t="s">
+      <c r="G24" s="69" t="s">
         <v>249</v>
       </c>
-      <c r="H24" s="67" t="s">
+      <c r="H24" s="69" t="s">
         <v>288</v>
       </c>
-      <c r="I24" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J24" s="67" t="s">
+      <c r="I24" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J24" s="69" t="s">
         <v>361</v>
       </c>
-      <c r="K24" s="68" t="s">
+      <c r="K24" s="70" t="s">
         <v>425</v>
       </c>
       <c r="L24" s="55">
@@ -3399,75 +3394,75 @@
         <v>1.28</v>
       </c>
     </row>
-    <row r="25" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="14"/>
       <c r="B25" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B25) - ROW($B$9)</f>
         <v>16</v>
       </c>
       <c r="C25" s="51">
         <v>4</v>
       </c>
-      <c r="D25" s="66" t="s">
+      <c r="D25" s="68" t="s">
         <v>56</v>
       </c>
-      <c r="E25" s="66" t="s">
+      <c r="E25" s="68" t="s">
         <v>125</v>
       </c>
-      <c r="F25" s="66" t="s">
+      <c r="F25" s="68" t="s">
         <v>190</v>
       </c>
-      <c r="G25" s="66" t="s">
+      <c r="G25" s="68" t="s">
         <v>250</v>
       </c>
-      <c r="H25" s="66" t="s">
+      <c r="H25" s="68" t="s">
         <v>289</v>
       </c>
-      <c r="I25" s="66" t="s">
+      <c r="I25" s="68" t="s">
         <v>344</v>
       </c>
-      <c r="J25" s="66" t="s">
+      <c r="J25" s="68" t="s">
         <v>362</v>
       </c>
-      <c r="K25" s="69" t="s">
+      <c r="K25" s="71" t="s">
         <v>426</v>
       </c>
       <c r="L25" s="57">
-        <f t="shared" ref="L25" si="8">C25*K25</f>
+        <f t="shared" ref="L25" si="7">C25*K25</f>
         <v>3.72</v>
       </c>
     </row>
     <row r="26" spans="1:12" s="3" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A26" s="14"/>
       <c r="B26" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B26) - ROW($B$9)</f>
         <v>17</v>
       </c>
       <c r="C26" s="50">
         <v>1</v>
       </c>
-      <c r="D26" s="65" t="s">
+      <c r="D26" s="67" t="s">
         <v>57</v>
       </c>
-      <c r="E26" s="65" t="s">
+      <c r="E26" s="67" t="s">
         <v>126</v>
       </c>
-      <c r="F26" s="67" t="s">
+      <c r="F26" s="69" t="s">
         <v>191</v>
       </c>
-      <c r="G26" s="67" t="s">
+      <c r="G26" s="69" t="s">
         <v>251</v>
       </c>
-      <c r="H26" s="67" t="s">
+      <c r="H26" s="69" t="s">
         <v>290</v>
       </c>
-      <c r="I26" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J26" s="67" t="s">
+      <c r="I26" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J26" s="69" t="s">
         <v>363</v>
       </c>
-      <c r="K26" s="68" t="s">
+      <c r="K26" s="70" t="s">
         <v>427</v>
       </c>
       <c r="L26" s="55">
@@ -3475,75 +3470,75 @@
         <v>2.2999999999999998</v>
       </c>
     </row>
-    <row r="27" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A27" s="14"/>
       <c r="B27" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B27) - ROW($B$9)</f>
         <v>18</v>
       </c>
       <c r="C27" s="51">
         <v>1</v>
       </c>
-      <c r="D27" s="66" t="s">
+      <c r="D27" s="68" t="s">
         <v>58</v>
       </c>
-      <c r="E27" s="66" t="s">
+      <c r="E27" s="68" t="s">
         <v>127</v>
       </c>
-      <c r="F27" s="66" t="s">
+      <c r="F27" s="68" t="s">
         <v>192</v>
       </c>
-      <c r="G27" s="66" t="s">
+      <c r="G27" s="68" t="s">
         <v>252</v>
       </c>
-      <c r="H27" s="66" t="s">
+      <c r="H27" s="68" t="s">
         <v>291</v>
       </c>
-      <c r="I27" s="66" t="s">
+      <c r="I27" s="68" t="s">
         <v>344</v>
       </c>
-      <c r="J27" s="66" t="s">
+      <c r="J27" s="68" t="s">
         <v>364</v>
       </c>
-      <c r="K27" s="69" t="s">
+      <c r="K27" s="71" t="s">
         <v>428</v>
       </c>
       <c r="L27" s="57">
-        <f t="shared" ref="L27" si="9">C27*K27</f>
+        <f t="shared" ref="L27" si="8">C27*K27</f>
         <v>7.0000000000000007E-2</v>
       </c>
     </row>
     <row r="28" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="14"/>
       <c r="B28" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B28) - ROW($B$9)</f>
         <v>19</v>
       </c>
       <c r="C28" s="50">
         <v>1</v>
       </c>
-      <c r="D28" s="65" t="s">
+      <c r="D28" s="67" t="s">
         <v>59</v>
       </c>
-      <c r="E28" s="65" t="s">
+      <c r="E28" s="67" t="s">
         <v>128</v>
       </c>
-      <c r="F28" s="67" t="s">
+      <c r="F28" s="69" t="s">
         <v>193</v>
       </c>
-      <c r="G28" s="67" t="s">
+      <c r="G28" s="69" t="s">
         <v>253</v>
       </c>
-      <c r="H28" s="67" t="s">
+      <c r="H28" s="69" t="s">
         <v>292</v>
       </c>
-      <c r="I28" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J28" s="67" t="s">
+      <c r="I28" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J28" s="69" t="s">
         <v>365</v>
       </c>
-      <c r="K28" s="68" t="s">
+      <c r="K28" s="70" t="s">
         <v>429</v>
       </c>
       <c r="L28" s="55">
@@ -3551,75 +3546,75 @@
         <v>1.4</v>
       </c>
     </row>
-    <row r="29" spans="1:12" s="3" customFormat="1" ht="56.25" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A29" s="14"/>
       <c r="B29" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B29) - ROW($B$9)</f>
         <v>20</v>
       </c>
       <c r="C29" s="51">
         <v>4</v>
       </c>
-      <c r="D29" s="66" t="s">
+      <c r="D29" s="68" t="s">
         <v>60</v>
       </c>
-      <c r="E29" s="66" t="s">
+      <c r="E29" s="68" t="s">
         <v>129</v>
       </c>
-      <c r="F29" s="66" t="s">
+      <c r="F29" s="68" t="s">
         <v>194</v>
       </c>
-      <c r="G29" s="66" t="s">
+      <c r="G29" s="68" t="s">
         <v>252</v>
       </c>
-      <c r="H29" s="66" t="s">
+      <c r="H29" s="68" t="s">
         <v>293</v>
       </c>
-      <c r="I29" s="66" t="s">
+      <c r="I29" s="68" t="s">
         <v>344</v>
       </c>
-      <c r="J29" s="66" t="s">
+      <c r="J29" s="68" t="s">
         <v>366</v>
       </c>
-      <c r="K29" s="69" t="s">
+      <c r="K29" s="71" t="s">
         <v>428</v>
       </c>
       <c r="L29" s="57">
-        <f t="shared" ref="L29" si="10">C29*K29</f>
+        <f t="shared" ref="L29" si="9">C29*K29</f>
         <v>0.28000000000000003</v>
       </c>
     </row>
     <row r="30" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="14"/>
       <c r="B30" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B30) - ROW($B$9)</f>
         <v>21</v>
       </c>
       <c r="C30" s="50">
         <v>1</v>
       </c>
-      <c r="D30" s="65" t="s">
+      <c r="D30" s="67" t="s">
         <v>61</v>
       </c>
-      <c r="E30" s="65" t="s">
+      <c r="E30" s="67" t="s">
         <v>129</v>
       </c>
-      <c r="F30" s="67" t="s">
+      <c r="F30" s="69" t="s">
         <v>195</v>
       </c>
-      <c r="G30" s="67" t="s">
+      <c r="G30" s="69" t="s">
         <v>254</v>
       </c>
-      <c r="H30" s="67" t="s">
+      <c r="H30" s="69" t="s">
         <v>294</v>
       </c>
-      <c r="I30" s="67" t="s">
+      <c r="I30" s="69" t="s">
         <v>344</v>
       </c>
-      <c r="J30" s="67" t="s">
+      <c r="J30" s="69" t="s">
         <v>367</v>
       </c>
-      <c r="K30" s="68" t="s">
+      <c r="K30" s="70" t="s">
         <v>430</v>
       </c>
       <c r="L30" s="55">
@@ -3627,75 +3622,75 @@
         <v>1.1000000000000001</v>
       </c>
     </row>
-    <row r="31" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A31" s="14"/>
       <c r="B31" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B31) - ROW($B$9)</f>
         <v>22</v>
       </c>
       <c r="C31" s="51">
         <v>1</v>
       </c>
-      <c r="D31" s="66" t="s">
+      <c r="D31" s="68" t="s">
         <v>62</v>
       </c>
-      <c r="E31" s="66" t="s">
+      <c r="E31" s="68" t="s">
         <v>130</v>
       </c>
-      <c r="F31" s="66" t="s">
+      <c r="F31" s="68" t="s">
         <v>196</v>
       </c>
-      <c r="G31" s="66" t="s">
+      <c r="G31" s="68" t="s">
         <v>255</v>
       </c>
-      <c r="H31" s="66" t="s">
+      <c r="H31" s="68" t="s">
         <v>295</v>
       </c>
-      <c r="I31" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J31" s="66" t="s">
+      <c r="I31" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J31" s="68" t="s">
         <v>368</v>
       </c>
-      <c r="K31" s="69" t="s">
+      <c r="K31" s="71" t="s">
         <v>431</v>
       </c>
       <c r="L31" s="57">
-        <f t="shared" ref="L31" si="11">C31*K31</f>
+        <f t="shared" ref="L31" si="10">C31*K31</f>
         <v>1.8</v>
       </c>
     </row>
     <row r="32" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="14"/>
       <c r="B32" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B32) - ROW($B$9)</f>
         <v>23</v>
       </c>
       <c r="C32" s="50">
         <v>1</v>
       </c>
-      <c r="D32" s="65" t="s">
+      <c r="D32" s="67" t="s">
         <v>63</v>
       </c>
-      <c r="E32" s="65" t="s">
+      <c r="E32" s="67" t="s">
         <v>131</v>
       </c>
-      <c r="F32" s="67" t="s">
+      <c r="F32" s="69" t="s">
         <v>197</v>
       </c>
-      <c r="G32" s="67" t="s">
+      <c r="G32" s="69" t="s">
         <v>256</v>
       </c>
-      <c r="H32" s="67" t="s">
+      <c r="H32" s="69" t="s">
         <v>296</v>
       </c>
-      <c r="I32" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J32" s="67" t="s">
+      <c r="I32" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J32" s="69" t="s">
         <v>369</v>
       </c>
-      <c r="K32" s="68" t="s">
+      <c r="K32" s="70" t="s">
         <v>432</v>
       </c>
       <c r="L32" s="55">
@@ -3703,75 +3698,75 @@
         <v>0.26</v>
       </c>
     </row>
-    <row r="33" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="14"/>
       <c r="B33" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B33) - ROW($B$9)</f>
         <v>24</v>
       </c>
       <c r="C33" s="51">
         <v>5</v>
       </c>
-      <c r="D33" s="66" t="s">
+      <c r="D33" s="68" t="s">
         <v>64</v>
       </c>
-      <c r="E33" s="66" t="s">
+      <c r="E33" s="68" t="s">
         <v>132</v>
       </c>
-      <c r="F33" s="66" t="s">
+      <c r="F33" s="68" t="s">
         <v>198</v>
       </c>
-      <c r="G33" s="66" t="s">
+      <c r="G33" s="68" t="s">
         <v>257</v>
       </c>
-      <c r="H33" s="66" t="s">
+      <c r="H33" s="68" t="s">
         <v>297</v>
       </c>
-      <c r="I33" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J33" s="66" t="s">
+      <c r="I33" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J33" s="68" t="s">
         <v>370</v>
       </c>
-      <c r="K33" s="69" t="s">
+      <c r="K33" s="71" t="s">
         <v>423</v>
       </c>
       <c r="L33" s="57">
-        <f t="shared" ref="L33" si="12">C33*K33</f>
+        <f t="shared" ref="L33" si="11">C33*K33</f>
         <v>0.5</v>
       </c>
     </row>
     <row r="34" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="14"/>
       <c r="B34" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B34) - ROW($B$9)</f>
         <v>25</v>
       </c>
       <c r="C34" s="50">
         <v>2</v>
       </c>
-      <c r="D34" s="65" t="s">
+      <c r="D34" s="67" t="s">
         <v>65</v>
       </c>
-      <c r="E34" s="65" t="s">
+      <c r="E34" s="67" t="s">
         <v>133</v>
       </c>
-      <c r="F34" s="67" t="s">
+      <c r="F34" s="69" t="s">
         <v>199</v>
       </c>
-      <c r="G34" s="67" t="s">
+      <c r="G34" s="69" t="s">
         <v>257</v>
       </c>
-      <c r="H34" s="67" t="s">
+      <c r="H34" s="69" t="s">
         <v>298</v>
       </c>
-      <c r="I34" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J34" s="67" t="s">
+      <c r="I34" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J34" s="69" t="s">
         <v>371</v>
       </c>
-      <c r="K34" s="68" t="s">
+      <c r="K34" s="70" t="s">
         <v>433</v>
       </c>
       <c r="L34" s="55">
@@ -3779,75 +3774,75 @@
         <v>0.3</v>
       </c>
     </row>
-    <row r="35" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="14"/>
       <c r="B35" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B35) - ROW($B$9)</f>
         <v>26</v>
       </c>
       <c r="C35" s="51">
         <v>1</v>
       </c>
-      <c r="D35" s="66" t="s">
+      <c r="D35" s="68" t="s">
         <v>66</v>
       </c>
-      <c r="E35" s="66" t="s">
+      <c r="E35" s="68" t="s">
         <v>134</v>
       </c>
-      <c r="F35" s="66" t="s">
+      <c r="F35" s="68" t="s">
         <v>200</v>
       </c>
-      <c r="G35" s="66" t="s">
+      <c r="G35" s="68" t="s">
         <v>257</v>
       </c>
-      <c r="H35" s="66" t="s">
+      <c r="H35" s="68" t="s">
         <v>299</v>
       </c>
-      <c r="I35" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J35" s="66" t="s">
+      <c r="I35" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J35" s="68" t="s">
         <v>372</v>
       </c>
-      <c r="K35" s="69" t="s">
+      <c r="K35" s="71" t="s">
         <v>434</v>
       </c>
       <c r="L35" s="57">
-        <f t="shared" ref="L35" si="13">C35*K35</f>
+        <f t="shared" ref="L35" si="12">C35*K35</f>
         <v>0.18</v>
       </c>
     </row>
     <row r="36" spans="1:12" s="3" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A36" s="14"/>
       <c r="B36" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B36) - ROW($B$9)</f>
         <v>27</v>
       </c>
       <c r="C36" s="50">
         <v>4</v>
       </c>
-      <c r="D36" s="65" t="s">
+      <c r="D36" s="67" t="s">
         <v>67</v>
       </c>
-      <c r="E36" s="65" t="s">
+      <c r="E36" s="67" t="s">
         <v>135</v>
       </c>
-      <c r="F36" s="67" t="s">
+      <c r="F36" s="69" t="s">
         <v>201</v>
       </c>
-      <c r="G36" s="67" t="s">
+      <c r="G36" s="69" t="s">
         <v>258</v>
       </c>
-      <c r="H36" s="67" t="s">
+      <c r="H36" s="69" t="s">
         <v>300</v>
       </c>
-      <c r="I36" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J36" s="67" t="s">
+      <c r="I36" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J36" s="69" t="s">
         <v>373</v>
       </c>
-      <c r="K36" s="68" t="s">
+      <c r="K36" s="70" t="s">
         <v>435</v>
       </c>
       <c r="L36" s="55">
@@ -3855,75 +3850,75 @@
         <v>2.3199999999999998</v>
       </c>
     </row>
-    <row r="37" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A37" s="14"/>
       <c r="B37" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B37) - ROW($B$9)</f>
         <v>28</v>
       </c>
       <c r="C37" s="51">
         <v>4</v>
       </c>
-      <c r="D37" s="66" t="s">
+      <c r="D37" s="68" t="s">
         <v>68</v>
       </c>
-      <c r="E37" s="66" t="s">
+      <c r="E37" s="68" t="s">
         <v>136</v>
       </c>
-      <c r="F37" s="66" t="s">
+      <c r="F37" s="68" t="s">
         <v>202</v>
       </c>
-      <c r="G37" s="66" t="s">
+      <c r="G37" s="68" t="s">
         <v>254</v>
       </c>
-      <c r="H37" s="66" t="s">
+      <c r="H37" s="68" t="s">
         <v>301</v>
       </c>
-      <c r="I37" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J37" s="66" t="s">
+      <c r="I37" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J37" s="68" t="s">
         <v>374</v>
       </c>
-      <c r="K37" s="69" t="s">
+      <c r="K37" s="71" t="s">
         <v>436</v>
       </c>
       <c r="L37" s="57">
-        <f t="shared" ref="L37" si="14">C37*K37</f>
+        <f t="shared" ref="L37" si="13">C37*K37</f>
         <v>5.44</v>
       </c>
     </row>
     <row r="38" spans="1:12" s="3" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A38" s="14"/>
       <c r="B38" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B38) - ROW($B$9)</f>
         <v>29</v>
       </c>
       <c r="C38" s="50">
         <v>1</v>
       </c>
-      <c r="D38" s="65" t="s">
+      <c r="D38" s="67" t="s">
         <v>69</v>
       </c>
-      <c r="E38" s="65" t="s">
+      <c r="E38" s="67" t="s">
         <v>137</v>
       </c>
-      <c r="F38" s="67" t="s">
+      <c r="F38" s="69" t="s">
         <v>203</v>
       </c>
-      <c r="G38" s="67" t="s">
+      <c r="G38" s="69" t="s">
         <v>259</v>
       </c>
-      <c r="H38" s="67" t="s">
+      <c r="H38" s="69" t="s">
         <v>302</v>
       </c>
-      <c r="I38" s="67" t="s">
+      <c r="I38" s="69" t="s">
         <v>259</v>
       </c>
-      <c r="J38" s="67" t="s">
+      <c r="J38" s="69" t="s">
         <v>302</v>
       </c>
-      <c r="K38" s="68" t="s">
+      <c r="K38" s="70" t="s">
         <v>437</v>
       </c>
       <c r="L38" s="55">
@@ -3931,75 +3926,75 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="39" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="14"/>
       <c r="B39" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B39) - ROW($B$9)</f>
         <v>30</v>
       </c>
       <c r="C39" s="51">
         <v>1</v>
       </c>
-      <c r="D39" s="66" t="s">
+      <c r="D39" s="68" t="s">
         <v>70</v>
       </c>
-      <c r="E39" s="66" t="s">
+      <c r="E39" s="68" t="s">
         <v>138</v>
       </c>
-      <c r="F39" s="66" t="s">
+      <c r="F39" s="68" t="s">
         <v>204</v>
       </c>
-      <c r="G39" s="66" t="s">
+      <c r="G39" s="68" t="s">
         <v>260</v>
       </c>
-      <c r="H39" s="66" t="s">
+      <c r="H39" s="68" t="s">
         <v>303</v>
       </c>
-      <c r="I39" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J39" s="66" t="s">
+      <c r="I39" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J39" s="68" t="s">
         <v>375</v>
       </c>
-      <c r="K39" s="69" t="s">
+      <c r="K39" s="71" t="s">
         <v>438</v>
       </c>
       <c r="L39" s="57">
-        <f t="shared" ref="L39" si="15">C39*K39</f>
+        <f t="shared" ref="L39" si="14">C39*K39</f>
         <v>299</v>
       </c>
     </row>
     <row r="40" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="14"/>
       <c r="B40" s="48">
-        <f t="shared" si="0"/>
+        <f>ROW(B40) - ROW($B$9)</f>
         <v>31</v>
       </c>
       <c r="C40" s="50">
         <v>2</v>
       </c>
-      <c r="D40" s="65" t="s">
+      <c r="D40" s="67" t="s">
         <v>71</v>
       </c>
-      <c r="E40" s="65" t="s">
+      <c r="E40" s="67" t="s">
         <v>139</v>
       </c>
-      <c r="F40" s="67" t="s">
+      <c r="F40" s="69" t="s">
         <v>205</v>
       </c>
-      <c r="G40" s="67" t="s">
+      <c r="G40" s="69" t="s">
         <v>249</v>
       </c>
-      <c r="H40" s="67" t="s">
+      <c r="H40" s="69" t="s">
         <v>304</v>
       </c>
-      <c r="I40" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J40" s="67" t="s">
+      <c r="I40" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J40" s="69" t="s">
         <v>376</v>
       </c>
-      <c r="K40" s="68" t="s">
+      <c r="K40" s="70" t="s">
         <v>439</v>
       </c>
       <c r="L40" s="55">
@@ -4007,75 +4002,75 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="41" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A41" s="14"/>
       <c r="B41" s="49">
-        <f t="shared" si="0"/>
+        <f>ROW(B41) - ROW($B$9)</f>
         <v>32</v>
       </c>
       <c r="C41" s="51">
         <v>2</v>
       </c>
-      <c r="D41" s="66" t="s">
+      <c r="D41" s="68" t="s">
         <v>72</v>
       </c>
-      <c r="E41" s="66" t="s">
+      <c r="E41" s="68" t="s">
         <v>140</v>
       </c>
-      <c r="F41" s="66" t="s">
+      <c r="F41" s="68" t="s">
         <v>206</v>
       </c>
-      <c r="G41" s="66" t="s">
+      <c r="G41" s="68" t="s">
         <v>261</v>
       </c>
-      <c r="H41" s="66" t="s">
+      <c r="H41" s="68" t="s">
         <v>305</v>
       </c>
-      <c r="I41" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J41" s="66" t="s">
+      <c r="I41" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J41" s="68" t="s">
         <v>377</v>
       </c>
-      <c r="K41" s="69" t="s">
+      <c r="K41" s="71" t="s">
         <v>440</v>
       </c>
       <c r="L41" s="57">
-        <f t="shared" ref="L41" si="16">C41*K41</f>
+        <f t="shared" ref="L41" si="15">C41*K41</f>
         <v>0.9</v>
       </c>
     </row>
     <row r="42" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="14"/>
       <c r="B42" s="48">
-        <f t="shared" ref="B42:B77" si="17">ROW(B42) - ROW($B$9)</f>
+        <f>ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
       <c r="C42" s="50">
         <v>8</v>
       </c>
-      <c r="D42" s="65" t="s">
+      <c r="D42" s="67" t="s">
         <v>73</v>
       </c>
-      <c r="E42" s="65" t="s">
+      <c r="E42" s="67" t="s">
         <v>141</v>
       </c>
-      <c r="F42" s="67" t="s">
+      <c r="F42" s="69" t="s">
         <v>207</v>
       </c>
-      <c r="G42" s="67" t="s">
+      <c r="G42" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H42" s="67" t="s">
+      <c r="H42" s="69" t="s">
         <v>306</v>
       </c>
-      <c r="I42" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J42" s="67" t="s">
+      <c r="I42" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J42" s="69" t="s">
         <v>378</v>
       </c>
-      <c r="K42" s="68" t="s">
+      <c r="K42" s="70" t="s">
         <v>415</v>
       </c>
       <c r="L42" s="55">
@@ -4083,75 +4078,75 @@
         <v>0.8</v>
       </c>
     </row>
-    <row r="43" spans="1:12" s="3" customFormat="1" ht="45" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A43" s="14"/>
       <c r="B43" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B43) - ROW($B$9)</f>
         <v>34</v>
       </c>
       <c r="C43" s="51">
         <v>26</v>
       </c>
-      <c r="D43" s="66" t="s">
+      <c r="D43" s="68" t="s">
         <v>74</v>
       </c>
-      <c r="E43" s="66" t="s">
+      <c r="E43" s="68" t="s">
         <v>142</v>
       </c>
-      <c r="F43" s="66" t="s">
+      <c r="F43" s="68" t="s">
         <v>208</v>
       </c>
-      <c r="G43" s="66" t="s">
+      <c r="G43" s="68" t="s">
         <v>246</v>
       </c>
-      <c r="H43" s="66" t="s">
+      <c r="H43" s="68" t="s">
         <v>307</v>
       </c>
-      <c r="I43" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J43" s="66" t="s">
+      <c r="I43" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J43" s="68" t="s">
         <v>379</v>
       </c>
-      <c r="K43" s="69" t="s">
+      <c r="K43" s="71" t="s">
         <v>423</v>
       </c>
       <c r="L43" s="57">
-        <f t="shared" ref="L43" si="18">C43*K43</f>
+        <f t="shared" ref="L43" si="16">C43*K43</f>
         <v>2.6</v>
       </c>
     </row>
     <row r="44" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="14"/>
       <c r="B44" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B44) - ROW($B$9)</f>
         <v>35</v>
       </c>
       <c r="C44" s="50">
         <v>1</v>
       </c>
-      <c r="D44" s="65" t="s">
+      <c r="D44" s="67" t="s">
         <v>75</v>
       </c>
-      <c r="E44" s="65" t="s">
+      <c r="E44" s="67" t="s">
         <v>143</v>
       </c>
-      <c r="F44" s="67" t="s">
+      <c r="F44" s="69" t="s">
         <v>209</v>
       </c>
-      <c r="G44" s="67" t="s">
+      <c r="G44" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H44" s="67" t="s">
+      <c r="H44" s="69" t="s">
         <v>308</v>
       </c>
-      <c r="I44" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J44" s="67" t="s">
+      <c r="I44" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J44" s="69" t="s">
         <v>380</v>
       </c>
-      <c r="K44" s="68" t="s">
+      <c r="K44" s="70" t="s">
         <v>415</v>
       </c>
       <c r="L44" s="55">
@@ -4159,75 +4154,75 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="45" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A45" s="14"/>
       <c r="B45" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B45) - ROW($B$9)</f>
         <v>36</v>
       </c>
       <c r="C45" s="51">
         <v>1</v>
       </c>
-      <c r="D45" s="66" t="s">
+      <c r="D45" s="68" t="s">
         <v>76</v>
       </c>
-      <c r="E45" s="66" t="s">
+      <c r="E45" s="68" t="s">
         <v>144</v>
       </c>
-      <c r="F45" s="66" t="s">
+      <c r="F45" s="68" t="s">
         <v>210</v>
       </c>
-      <c r="G45" s="66" t="s">
+      <c r="G45" s="68" t="s">
         <v>246</v>
       </c>
-      <c r="H45" s="66" t="s">
+      <c r="H45" s="68" t="s">
         <v>309</v>
       </c>
-      <c r="I45" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J45" s="66" t="s">
+      <c r="I45" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J45" s="68" t="s">
         <v>381</v>
       </c>
-      <c r="K45" s="69" t="s">
+      <c r="K45" s="71" t="s">
         <v>415</v>
       </c>
       <c r="L45" s="57">
-        <f t="shared" ref="L45" si="19">C45*K45</f>
+        <f t="shared" ref="L45" si="17">C45*K45</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="46" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="14"/>
       <c r="B46" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B46) - ROW($B$9)</f>
         <v>37</v>
       </c>
       <c r="C46" s="50">
         <v>4</v>
       </c>
-      <c r="D46" s="65" t="s">
+      <c r="D46" s="67" t="s">
         <v>77</v>
       </c>
-      <c r="E46" s="65" t="s">
+      <c r="E46" s="67" t="s">
         <v>145</v>
       </c>
-      <c r="F46" s="67" t="s">
+      <c r="F46" s="69" t="s">
         <v>211</v>
       </c>
-      <c r="G46" s="67" t="s">
+      <c r="G46" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H46" s="67" t="s">
+      <c r="H46" s="69" t="s">
         <v>310</v>
       </c>
-      <c r="I46" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J46" s="67" t="s">
+      <c r="I46" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J46" s="69" t="s">
         <v>382</v>
       </c>
-      <c r="K46" s="68" t="s">
+      <c r="K46" s="70" t="s">
         <v>415</v>
       </c>
       <c r="L46" s="55">
@@ -4235,75 +4230,75 @@
         <v>0.4</v>
       </c>
     </row>
-    <row r="47" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A47" s="14"/>
       <c r="B47" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B47) - ROW($B$9)</f>
         <v>38</v>
       </c>
       <c r="C47" s="51">
         <v>2</v>
       </c>
-      <c r="D47" s="66" t="s">
+      <c r="D47" s="68" t="s">
         <v>78</v>
       </c>
-      <c r="E47" s="66" t="s">
+      <c r="E47" s="68" t="s">
         <v>146</v>
       </c>
-      <c r="F47" s="66" t="s">
+      <c r="F47" s="68" t="s">
         <v>212</v>
       </c>
-      <c r="G47" s="66" t="s">
+      <c r="G47" s="68" t="s">
         <v>246</v>
       </c>
-      <c r="H47" s="66" t="s">
+      <c r="H47" s="68" t="s">
         <v>311</v>
       </c>
-      <c r="I47" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J47" s="66" t="s">
+      <c r="I47" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J47" s="68" t="s">
         <v>383</v>
       </c>
-      <c r="K47" s="69" t="s">
+      <c r="K47" s="71" t="s">
         <v>425</v>
       </c>
       <c r="L47" s="57">
-        <f t="shared" ref="L47" si="20">C47*K47</f>
+        <f t="shared" ref="L47" si="18">C47*K47</f>
         <v>0.32</v>
       </c>
     </row>
     <row r="48" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="14"/>
       <c r="B48" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B48) - ROW($B$9)</f>
         <v>39</v>
       </c>
       <c r="C48" s="50">
         <v>2</v>
       </c>
-      <c r="D48" s="65" t="s">
+      <c r="D48" s="67" t="s">
         <v>79</v>
       </c>
-      <c r="E48" s="65" t="s">
+      <c r="E48" s="67" t="s">
         <v>147</v>
       </c>
-      <c r="F48" s="67" t="s">
+      <c r="F48" s="69" t="s">
         <v>213</v>
       </c>
-      <c r="G48" s="67" t="s">
+      <c r="G48" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H48" s="67" t="s">
+      <c r="H48" s="69" t="s">
         <v>312</v>
       </c>
-      <c r="I48" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J48" s="67" t="s">
+      <c r="I48" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J48" s="69" t="s">
         <v>384</v>
       </c>
-      <c r="K48" s="68" t="s">
+      <c r="K48" s="70" t="s">
         <v>423</v>
       </c>
       <c r="L48" s="55">
@@ -4311,75 +4306,75 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="49" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A49" s="14"/>
       <c r="B49" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B49) - ROW($B$9)</f>
         <v>40</v>
       </c>
       <c r="C49" s="51">
         <v>1</v>
       </c>
-      <c r="D49" s="66" t="s">
+      <c r="D49" s="68" t="s">
         <v>80</v>
       </c>
-      <c r="E49" s="66" t="s">
+      <c r="E49" s="68" t="s">
         <v>148</v>
       </c>
-      <c r="F49" s="66" t="s">
+      <c r="F49" s="68" t="s">
         <v>214</v>
       </c>
-      <c r="G49" s="66" t="s">
+      <c r="G49" s="68" t="s">
         <v>262</v>
       </c>
-      <c r="H49" s="66" t="s">
+      <c r="H49" s="68" t="s">
         <v>313</v>
       </c>
-      <c r="I49" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J49" s="66" t="s">
+      <c r="I49" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J49" s="68" t="s">
         <v>385</v>
       </c>
-      <c r="K49" s="69" t="s">
+      <c r="K49" s="71" t="s">
         <v>441</v>
       </c>
       <c r="L49" s="57">
-        <f t="shared" ref="L49" si="21">C49*K49</f>
+        <f t="shared" ref="L49" si="19">C49*K49</f>
         <v>2.56</v>
       </c>
     </row>
     <row r="50" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="14"/>
       <c r="B50" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B50) - ROW($B$9)</f>
         <v>41</v>
       </c>
       <c r="C50" s="50">
         <v>1</v>
       </c>
-      <c r="D50" s="65" t="s">
+      <c r="D50" s="67" t="s">
         <v>81</v>
       </c>
-      <c r="E50" s="65" t="s">
+      <c r="E50" s="67" t="s">
         <v>149</v>
       </c>
-      <c r="F50" s="67" t="s">
+      <c r="F50" s="69" t="s">
         <v>215</v>
       </c>
-      <c r="G50" s="67" t="s">
+      <c r="G50" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H50" s="67" t="s">
+      <c r="H50" s="69" t="s">
         <v>314</v>
       </c>
-      <c r="I50" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J50" s="67" t="s">
+      <c r="I50" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J50" s="69" t="s">
         <v>386</v>
       </c>
-      <c r="K50" s="68" t="s">
+      <c r="K50" s="70" t="s">
         <v>423</v>
       </c>
       <c r="L50" s="55">
@@ -4387,75 +4382,75 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="51" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A51" s="14"/>
       <c r="B51" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B51) - ROW($B$9)</f>
         <v>42</v>
       </c>
       <c r="C51" s="51">
         <v>2</v>
       </c>
-      <c r="D51" s="66" t="s">
+      <c r="D51" s="68" t="s">
         <v>82</v>
       </c>
-      <c r="E51" s="66" t="s">
+      <c r="E51" s="68" t="s">
         <v>150</v>
       </c>
-      <c r="F51" s="66" t="s">
+      <c r="F51" s="68" t="s">
         <v>216</v>
       </c>
-      <c r="G51" s="66" t="s">
+      <c r="G51" s="68" t="s">
         <v>246</v>
       </c>
-      <c r="H51" s="66" t="s">
+      <c r="H51" s="68" t="s">
         <v>315</v>
       </c>
-      <c r="I51" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J51" s="66" t="s">
+      <c r="I51" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J51" s="68" t="s">
         <v>387</v>
       </c>
-      <c r="K51" s="69" t="s">
+      <c r="K51" s="71" t="s">
         <v>415</v>
       </c>
       <c r="L51" s="57">
-        <f t="shared" ref="L51" si="22">C51*K51</f>
+        <f t="shared" ref="L51" si="20">C51*K51</f>
         <v>0.2</v>
       </c>
     </row>
     <row r="52" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="14"/>
       <c r="B52" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B52) - ROW($B$9)</f>
         <v>43</v>
       </c>
       <c r="C52" s="50">
         <v>6</v>
       </c>
-      <c r="D52" s="65" t="s">
+      <c r="D52" s="67" t="s">
         <v>83</v>
       </c>
-      <c r="E52" s="65" t="s">
+      <c r="E52" s="67" t="s">
         <v>151</v>
       </c>
-      <c r="F52" s="67" t="s">
+      <c r="F52" s="69" t="s">
         <v>217</v>
       </c>
-      <c r="G52" s="67" t="s">
+      <c r="G52" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H52" s="67" t="s">
+      <c r="H52" s="69" t="s">
         <v>316</v>
       </c>
-      <c r="I52" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J52" s="67" t="s">
+      <c r="I52" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J52" s="69" t="s">
         <v>388</v>
       </c>
-      <c r="K52" s="68" t="s">
+      <c r="K52" s="70" t="s">
         <v>415</v>
       </c>
       <c r="L52" s="55">
@@ -4463,75 +4458,75 @@
         <v>0.60000000000000009</v>
       </c>
     </row>
-    <row r="53" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A53" s="14"/>
       <c r="B53" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B53) - ROW($B$9)</f>
         <v>44</v>
       </c>
       <c r="C53" s="51">
         <v>1</v>
       </c>
-      <c r="D53" s="66" t="s">
+      <c r="D53" s="68" t="s">
         <v>84</v>
       </c>
-      <c r="E53" s="66" t="s">
+      <c r="E53" s="68" t="s">
         <v>152</v>
       </c>
-      <c r="F53" s="66" t="s">
+      <c r="F53" s="68" t="s">
         <v>218</v>
       </c>
-      <c r="G53" s="66" t="s">
+      <c r="G53" s="68" t="s">
         <v>262</v>
       </c>
-      <c r="H53" s="66" t="s">
+      <c r="H53" s="68" t="s">
         <v>317</v>
       </c>
-      <c r="I53" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J53" s="66" t="s">
+      <c r="I53" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J53" s="68" t="s">
         <v>389</v>
       </c>
-      <c r="K53" s="69" t="s">
+      <c r="K53" s="71" t="s">
         <v>442</v>
       </c>
       <c r="L53" s="57">
-        <f t="shared" ref="L53" si="23">C53*K53</f>
+        <f t="shared" ref="L53" si="21">C53*K53</f>
         <v>2.2000000000000002</v>
       </c>
     </row>
     <row r="54" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="14"/>
       <c r="B54" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B54) - ROW($B$9)</f>
         <v>45</v>
       </c>
       <c r="C54" s="50">
         <v>1</v>
       </c>
-      <c r="D54" s="65" t="s">
+      <c r="D54" s="67" t="s">
         <v>85</v>
       </c>
-      <c r="E54" s="65" t="s">
+      <c r="E54" s="67" t="s">
         <v>153</v>
       </c>
-      <c r="F54" s="67" t="s">
+      <c r="F54" s="69" t="s">
         <v>219</v>
       </c>
-      <c r="G54" s="67" t="s">
+      <c r="G54" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H54" s="67" t="s">
+      <c r="H54" s="69" t="s">
         <v>318</v>
       </c>
-      <c r="I54" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J54" s="67" t="s">
+      <c r="I54" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J54" s="69" t="s">
         <v>390</v>
       </c>
-      <c r="K54" s="68" t="s">
+      <c r="K54" s="70" t="s">
         <v>415</v>
       </c>
       <c r="L54" s="55">
@@ -4539,75 +4534,75 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="55" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A55" s="14"/>
       <c r="B55" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B55) - ROW($B$9)</f>
         <v>46</v>
       </c>
       <c r="C55" s="51">
         <v>1</v>
       </c>
-      <c r="D55" s="66" t="s">
+      <c r="D55" s="68" t="s">
         <v>86</v>
       </c>
-      <c r="E55" s="66" t="s">
+      <c r="E55" s="68" t="s">
         <v>154</v>
       </c>
-      <c r="F55" s="66" t="s">
+      <c r="F55" s="68" t="s">
         <v>220</v>
       </c>
-      <c r="G55" s="66" t="s">
+      <c r="G55" s="68" t="s">
         <v>246</v>
       </c>
-      <c r="H55" s="66" t="s">
+      <c r="H55" s="68" t="s">
         <v>319</v>
       </c>
-      <c r="I55" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J55" s="66" t="s">
+      <c r="I55" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J55" s="68" t="s">
         <v>391</v>
       </c>
-      <c r="K55" s="69" t="s">
+      <c r="K55" s="71" t="s">
         <v>423</v>
       </c>
       <c r="L55" s="57">
-        <f t="shared" ref="L55" si="24">C55*K55</f>
+        <f t="shared" ref="L55" si="22">C55*K55</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="56" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A56" s="14"/>
       <c r="B56" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B56) - ROW($B$9)</f>
         <v>47</v>
       </c>
       <c r="C56" s="50">
         <v>2</v>
       </c>
-      <c r="D56" s="65" t="s">
+      <c r="D56" s="67" t="s">
         <v>87</v>
       </c>
-      <c r="E56" s="65" t="s">
+      <c r="E56" s="67" t="s">
         <v>155</v>
       </c>
-      <c r="F56" s="67" t="s">
+      <c r="F56" s="69" t="s">
         <v>221</v>
       </c>
-      <c r="G56" s="67" t="s">
+      <c r="G56" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H56" s="67" t="s">
+      <c r="H56" s="69" t="s">
         <v>320</v>
       </c>
-      <c r="I56" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J56" s="67" t="s">
+      <c r="I56" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J56" s="69" t="s">
         <v>392</v>
       </c>
-      <c r="K56" s="68" t="s">
+      <c r="K56" s="70" t="s">
         <v>423</v>
       </c>
       <c r="L56" s="55">
@@ -4615,75 +4610,75 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="57" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A57" s="14"/>
       <c r="B57" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B57) - ROW($B$9)</f>
         <v>48</v>
       </c>
       <c r="C57" s="51">
         <v>7</v>
       </c>
-      <c r="D57" s="66" t="s">
+      <c r="D57" s="68" t="s">
         <v>88</v>
       </c>
-      <c r="E57" s="66" t="s">
+      <c r="E57" s="68" t="s">
         <v>156</v>
       </c>
-      <c r="F57" s="66" t="s">
+      <c r="F57" s="68" t="s">
         <v>222</v>
       </c>
-      <c r="G57" s="66" t="s">
+      <c r="G57" s="68" t="s">
         <v>246</v>
       </c>
-      <c r="H57" s="66" t="s">
+      <c r="H57" s="68" t="s">
         <v>321</v>
       </c>
-      <c r="I57" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J57" s="66" t="s">
+      <c r="I57" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J57" s="68" t="s">
         <v>393</v>
       </c>
-      <c r="K57" s="69" t="s">
+      <c r="K57" s="71" t="s">
         <v>417</v>
       </c>
       <c r="L57" s="57">
-        <f t="shared" ref="L57" si="25">C57*K57</f>
+        <f t="shared" ref="L57" si="23">C57*K57</f>
         <v>0.91</v>
       </c>
     </row>
     <row r="58" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="14"/>
       <c r="B58" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B58) - ROW($B$9)</f>
         <v>49</v>
       </c>
       <c r="C58" s="50">
         <v>1</v>
       </c>
-      <c r="D58" s="65" t="s">
+      <c r="D58" s="67" t="s">
         <v>89</v>
       </c>
-      <c r="E58" s="65" t="s">
+      <c r="E58" s="67" t="s">
         <v>157</v>
       </c>
-      <c r="F58" s="67" t="s">
+      <c r="F58" s="69" t="s">
         <v>223</v>
       </c>
-      <c r="G58" s="67" t="s">
+      <c r="G58" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H58" s="67" t="s">
+      <c r="H58" s="69" t="s">
         <v>322</v>
       </c>
-      <c r="I58" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J58" s="67" t="s">
+      <c r="I58" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J58" s="69" t="s">
         <v>394</v>
       </c>
-      <c r="K58" s="68" t="s">
+      <c r="K58" s="70" t="s">
         <v>415</v>
       </c>
       <c r="L58" s="55">
@@ -4691,75 +4686,75 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="59" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A59" s="14"/>
       <c r="B59" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B59) - ROW($B$9)</f>
         <v>50</v>
       </c>
       <c r="C59" s="51">
         <v>1</v>
       </c>
-      <c r="D59" s="66" t="s">
+      <c r="D59" s="68" t="s">
         <v>90</v>
       </c>
-      <c r="E59" s="66" t="s">
+      <c r="E59" s="68" t="s">
         <v>158</v>
       </c>
-      <c r="F59" s="66" t="s">
+      <c r="F59" s="68" t="s">
         <v>224</v>
       </c>
-      <c r="G59" s="66" t="s">
+      <c r="G59" s="68" t="s">
         <v>246</v>
       </c>
-      <c r="H59" s="66" t="s">
+      <c r="H59" s="68" t="s">
         <v>323</v>
       </c>
-      <c r="I59" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J59" s="66" t="s">
+      <c r="I59" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J59" s="68" t="s">
         <v>395</v>
       </c>
-      <c r="K59" s="69" t="s">
+      <c r="K59" s="71" t="s">
         <v>423</v>
       </c>
       <c r="L59" s="57">
-        <f t="shared" ref="L59" si="26">C59*K59</f>
+        <f t="shared" ref="L59" si="24">C59*K59</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="60" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="14"/>
       <c r="B60" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B60) - ROW($B$9)</f>
         <v>51</v>
       </c>
       <c r="C60" s="50">
         <v>1</v>
       </c>
-      <c r="D60" s="65" t="s">
+      <c r="D60" s="67" t="s">
         <v>91</v>
       </c>
-      <c r="E60" s="65" t="s">
+      <c r="E60" s="67" t="s">
         <v>159</v>
       </c>
-      <c r="F60" s="67" t="s">
+      <c r="F60" s="69" t="s">
         <v>225</v>
       </c>
-      <c r="G60" s="67" t="s">
+      <c r="G60" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H60" s="67" t="s">
+      <c r="H60" s="69" t="s">
         <v>324</v>
       </c>
-      <c r="I60" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J60" s="67" t="s">
+      <c r="I60" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J60" s="69" t="s">
         <v>396</v>
       </c>
-      <c r="K60" s="68" t="s">
+      <c r="K60" s="70" t="s">
         <v>423</v>
       </c>
       <c r="L60" s="55">
@@ -4767,75 +4762,75 @@
         <v>0.1</v>
       </c>
     </row>
-    <row r="61" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A61" s="14"/>
       <c r="B61" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B61) - ROW($B$9)</f>
         <v>52</v>
       </c>
       <c r="C61" s="51">
         <v>1</v>
       </c>
-      <c r="D61" s="66" t="s">
+      <c r="D61" s="68" t="s">
         <v>92</v>
       </c>
-      <c r="E61" s="66" t="s">
+      <c r="E61" s="68" t="s">
         <v>160</v>
       </c>
-      <c r="F61" s="66" t="s">
+      <c r="F61" s="68" t="s">
         <v>226</v>
       </c>
-      <c r="G61" s="66" t="s">
+      <c r="G61" s="68" t="s">
         <v>246</v>
       </c>
-      <c r="H61" s="66" t="s">
+      <c r="H61" s="68" t="s">
         <v>325</v>
       </c>
-      <c r="I61" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J61" s="66" t="s">
+      <c r="I61" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J61" s="68" t="s">
         <v>397</v>
       </c>
-      <c r="K61" s="69" t="s">
+      <c r="K61" s="71" t="s">
         <v>423</v>
       </c>
       <c r="L61" s="57">
-        <f t="shared" ref="L61" si="27">C61*K61</f>
+        <f t="shared" ref="L61" si="25">C61*K61</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="62" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="14"/>
       <c r="B62" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B62) - ROW($B$9)</f>
         <v>53</v>
       </c>
       <c r="C62" s="50">
         <v>1</v>
       </c>
-      <c r="D62" s="65" t="s">
+      <c r="D62" s="67" t="s">
         <v>93</v>
       </c>
-      <c r="E62" s="65" t="s">
+      <c r="E62" s="67" t="s">
         <v>161</v>
       </c>
-      <c r="F62" s="67" t="s">
+      <c r="F62" s="69" t="s">
         <v>227</v>
       </c>
-      <c r="G62" s="67" t="s">
+      <c r="G62" s="69" t="s">
         <v>246</v>
       </c>
-      <c r="H62" s="67" t="s">
+      <c r="H62" s="69" t="s">
         <v>326</v>
       </c>
-      <c r="I62" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J62" s="67" t="s">
+      <c r="I62" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J62" s="69" t="s">
         <v>398</v>
       </c>
-      <c r="K62" s="68" t="s">
+      <c r="K62" s="70" t="s">
         <v>419</v>
       </c>
       <c r="L62" s="55">
@@ -4843,75 +4838,75 @@
         <v>0.12</v>
       </c>
     </row>
-    <row r="63" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A63" s="14"/>
       <c r="B63" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B63) - ROW($B$9)</f>
         <v>54</v>
       </c>
       <c r="C63" s="51">
         <v>1</v>
       </c>
-      <c r="D63" s="66" t="s">
+      <c r="D63" s="68" t="s">
         <v>94</v>
       </c>
-      <c r="E63" s="66" t="s">
+      <c r="E63" s="68" t="s">
         <v>162</v>
       </c>
-      <c r="F63" s="66" t="s">
+      <c r="F63" s="68" t="s">
         <v>228</v>
       </c>
-      <c r="G63" s="66" t="s">
+      <c r="G63" s="68" t="s">
         <v>246</v>
       </c>
-      <c r="H63" s="66" t="s">
+      <c r="H63" s="68" t="s">
         <v>327</v>
       </c>
-      <c r="I63" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J63" s="66" t="s">
+      <c r="I63" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J63" s="68" t="s">
         <v>399</v>
       </c>
-      <c r="K63" s="69" t="s">
+      <c r="K63" s="71" t="s">
         <v>423</v>
       </c>
       <c r="L63" s="57">
-        <f t="shared" ref="L63" si="28">C63*K63</f>
+        <f t="shared" ref="L63" si="26">C63*K63</f>
         <v>0.1</v>
       </c>
     </row>
     <row r="64" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A64" s="14"/>
       <c r="B64" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B64) - ROW($B$9)</f>
         <v>55</v>
       </c>
       <c r="C64" s="50">
         <v>1</v>
       </c>
-      <c r="D64" s="65" t="s">
+      <c r="D64" s="67" t="s">
         <v>95</v>
       </c>
-      <c r="E64" s="65" t="s">
+      <c r="E64" s="67" t="s">
         <v>124</v>
       </c>
-      <c r="F64" s="67" t="s">
+      <c r="F64" s="69" t="s">
         <v>229</v>
       </c>
-      <c r="G64" s="67" t="s">
+      <c r="G64" s="69" t="s">
         <v>263</v>
       </c>
-      <c r="H64" s="67" t="s">
+      <c r="H64" s="69" t="s">
         <v>328</v>
       </c>
-      <c r="I64" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J64" s="67" t="s">
+      <c r="I64" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J64" s="69" t="s">
         <v>400</v>
       </c>
-      <c r="K64" s="68" t="s">
+      <c r="K64" s="70" t="s">
         <v>443</v>
       </c>
       <c r="L64" s="55">
@@ -4919,75 +4914,75 @@
         <v>3.77</v>
       </c>
     </row>
-    <row r="65" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A65" s="14"/>
       <c r="B65" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B65) - ROW($B$9)</f>
         <v>56</v>
       </c>
       <c r="C65" s="51">
         <v>1</v>
       </c>
-      <c r="D65" s="66" t="s">
+      <c r="D65" s="68" t="s">
         <v>96</v>
       </c>
-      <c r="E65" s="66" t="s">
+      <c r="E65" s="68" t="s">
         <v>163</v>
       </c>
-      <c r="F65" s="66" t="s">
+      <c r="F65" s="68" t="s">
         <v>230</v>
       </c>
-      <c r="G65" s="66" t="s">
+      <c r="G65" s="68" t="s">
         <v>264</v>
       </c>
-      <c r="H65" s="66" t="s">
+      <c r="H65" s="68" t="s">
         <v>329</v>
       </c>
-      <c r="I65" s="66" t="s">
+      <c r="I65" s="68" t="s">
         <v>344</v>
       </c>
-      <c r="J65" s="66" t="s">
+      <c r="J65" s="68" t="s">
         <v>329</v>
       </c>
-      <c r="K65" s="69" t="s">
+      <c r="K65" s="71" t="s">
         <v>444</v>
       </c>
       <c r="L65" s="57">
-        <f t="shared" ref="L65" si="29">C65*K65</f>
+        <f t="shared" ref="L65" si="27">C65*K65</f>
         <v>1</v>
       </c>
     </row>
     <row r="66" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A66" s="14"/>
       <c r="B66" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B66) - ROW($B$9)</f>
         <v>57</v>
       </c>
       <c r="C66" s="50">
         <v>5</v>
       </c>
-      <c r="D66" s="65" t="s">
+      <c r="D66" s="67" t="s">
         <v>97</v>
       </c>
-      <c r="E66" s="65" t="s">
+      <c r="E66" s="67" t="s">
         <v>164</v>
       </c>
-      <c r="F66" s="67" t="s">
+      <c r="F66" s="69" t="s">
         <v>231</v>
       </c>
-      <c r="G66" s="67" t="s">
+      <c r="G66" s="69" t="s">
         <v>265</v>
       </c>
-      <c r="H66" s="67" t="s">
+      <c r="H66" s="69" t="s">
         <v>330</v>
       </c>
-      <c r="I66" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J66" s="67" t="s">
+      <c r="I66" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J66" s="69" t="s">
         <v>401</v>
       </c>
-      <c r="K66" s="68" t="s">
+      <c r="K66" s="70" t="s">
         <v>445</v>
       </c>
       <c r="L66" s="55">
@@ -4995,75 +4990,75 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="67" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A67" s="14"/>
       <c r="B67" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B67) - ROW($B$9)</f>
         <v>58</v>
       </c>
       <c r="C67" s="51">
         <v>1</v>
       </c>
-      <c r="D67" s="66" t="s">
+      <c r="D67" s="68" t="s">
         <v>98</v>
       </c>
-      <c r="E67" s="66" t="s">
+      <c r="E67" s="68" t="s">
         <v>165</v>
       </c>
-      <c r="F67" s="66" t="s">
+      <c r="F67" s="68" t="s">
         <v>232</v>
       </c>
-      <c r="G67" s="66" t="s">
+      <c r="G67" s="68" t="s">
         <v>266</v>
       </c>
-      <c r="H67" s="66" t="s">
+      <c r="H67" s="68" t="s">
         <v>331</v>
       </c>
-      <c r="I67" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J67" s="66" t="s">
+      <c r="I67" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J67" s="68" t="s">
         <v>402</v>
       </c>
-      <c r="K67" s="69" t="s">
+      <c r="K67" s="71" t="s">
         <v>446</v>
       </c>
       <c r="L67" s="57">
-        <f t="shared" ref="L67" si="30">C67*K67</f>
+        <f t="shared" ref="L67" si="28">C67*K67</f>
         <v>0.48</v>
       </c>
     </row>
     <row r="68" spans="1:12" s="3" customFormat="1" ht="22.5" x14ac:dyDescent="0.2">
       <c r="A68" s="14"/>
       <c r="B68" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B68) - ROW($B$9)</f>
         <v>59</v>
       </c>
       <c r="C68" s="50">
         <v>8</v>
       </c>
-      <c r="D68" s="65" t="s">
+      <c r="D68" s="67" t="s">
         <v>99</v>
       </c>
-      <c r="E68" s="65" t="s">
+      <c r="E68" s="67" t="s">
         <v>166</v>
       </c>
-      <c r="F68" s="67" t="s">
+      <c r="F68" s="69" t="s">
         <v>233</v>
       </c>
-      <c r="G68" s="67" t="s">
+      <c r="G68" s="69" t="s">
         <v>267</v>
       </c>
-      <c r="H68" s="67" t="s">
+      <c r="H68" s="69" t="s">
         <v>332</v>
       </c>
-      <c r="I68" s="67" t="s">
+      <c r="I68" s="69" t="s">
         <v>344</v>
       </c>
-      <c r="J68" s="67" t="s">
+      <c r="J68" s="69" t="s">
         <v>403</v>
       </c>
-      <c r="K68" s="68" t="s">
+      <c r="K68" s="70" t="s">
         <v>414</v>
       </c>
       <c r="L68" s="55">
@@ -5071,75 +5066,75 @@
         <v>2.2400000000000002</v>
       </c>
     </row>
-    <row r="69" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A69" s="14"/>
       <c r="B69" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B69) - ROW($B$9)</f>
         <v>60</v>
       </c>
       <c r="C69" s="51">
         <v>2</v>
       </c>
-      <c r="D69" s="66" t="s">
+      <c r="D69" s="68" t="s">
         <v>100</v>
       </c>
-      <c r="E69" s="66" t="s">
+      <c r="E69" s="68" t="s">
         <v>167</v>
       </c>
-      <c r="F69" s="66" t="s">
+      <c r="F69" s="68" t="s">
         <v>234</v>
       </c>
-      <c r="G69" s="66" t="s">
+      <c r="G69" s="68" t="s">
         <v>268</v>
       </c>
-      <c r="H69" s="66" t="s">
+      <c r="H69" s="68" t="s">
         <v>333</v>
       </c>
-      <c r="I69" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J69" s="66" t="s">
+      <c r="I69" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J69" s="68" t="s">
         <v>404</v>
       </c>
-      <c r="K69" s="69" t="s">
+      <c r="K69" s="71" t="s">
         <v>447</v>
       </c>
       <c r="L69" s="57">
-        <f t="shared" ref="L69" si="31">C69*K69</f>
+        <f t="shared" ref="L69" si="29">C69*K69</f>
         <v>3.08</v>
       </c>
     </row>
     <row r="70" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A70" s="14"/>
       <c r="B70" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B70) - ROW($B$9)</f>
         <v>61</v>
       </c>
       <c r="C70" s="50">
         <v>1</v>
       </c>
-      <c r="D70" s="65" t="s">
+      <c r="D70" s="67" t="s">
         <v>101</v>
       </c>
-      <c r="E70" s="65" t="s">
+      <c r="E70" s="67" t="s">
         <v>168</v>
       </c>
-      <c r="F70" s="67" t="s">
+      <c r="F70" s="69" t="s">
         <v>235</v>
       </c>
-      <c r="G70" s="67" t="s">
+      <c r="G70" s="69" t="s">
         <v>269</v>
       </c>
-      <c r="H70" s="67" t="s">
+      <c r="H70" s="69" t="s">
         <v>334</v>
       </c>
-      <c r="I70" s="67" t="s">
+      <c r="I70" s="69" t="s">
         <v>345</v>
       </c>
-      <c r="J70" s="67" t="s">
+      <c r="J70" s="69" t="s">
         <v>405</v>
       </c>
-      <c r="K70" s="68" t="s">
+      <c r="K70" s="70" t="s">
         <v>448</v>
       </c>
       <c r="L70" s="55">
@@ -5147,75 +5142,75 @@
         <v>16.989999999999998</v>
       </c>
     </row>
-    <row r="71" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A71" s="14"/>
       <c r="B71" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B71) - ROW($B$9)</f>
         <v>62</v>
       </c>
       <c r="C71" s="51">
         <v>2</v>
       </c>
-      <c r="D71" s="66" t="s">
+      <c r="D71" s="68" t="s">
         <v>102</v>
       </c>
-      <c r="E71" s="66" t="s">
+      <c r="E71" s="68" t="s">
         <v>169</v>
       </c>
-      <c r="F71" s="66" t="s">
+      <c r="F71" s="68" t="s">
         <v>236</v>
       </c>
-      <c r="G71" s="66" t="s">
+      <c r="G71" s="68" t="s">
         <v>270</v>
       </c>
-      <c r="H71" s="66" t="s">
+      <c r="H71" s="68" t="s">
         <v>335</v>
       </c>
-      <c r="I71" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J71" s="66" t="s">
+      <c r="I71" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J71" s="68" t="s">
         <v>406</v>
       </c>
-      <c r="K71" s="69" t="s">
+      <c r="K71" s="71" t="s">
         <v>449</v>
       </c>
       <c r="L71" s="57">
-        <f t="shared" ref="L71" si="32">C71*K71</f>
+        <f t="shared" ref="L71" si="30">C71*K71</f>
         <v>24.04</v>
       </c>
     </row>
     <row r="72" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A72" s="14"/>
       <c r="B72" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B72) - ROW($B$9)</f>
         <v>63</v>
       </c>
       <c r="C72" s="50">
         <v>3</v>
       </c>
-      <c r="D72" s="65" t="s">
+      <c r="D72" s="67" t="s">
         <v>103</v>
       </c>
-      <c r="E72" s="65" t="s">
+      <c r="E72" s="67" t="s">
         <v>170</v>
       </c>
-      <c r="F72" s="67" t="s">
+      <c r="F72" s="69" t="s">
         <v>237</v>
       </c>
-      <c r="G72" s="67" t="s">
+      <c r="G72" s="69" t="s">
         <v>270</v>
       </c>
-      <c r="H72" s="67" t="s">
+      <c r="H72" s="69" t="s">
         <v>336</v>
       </c>
-      <c r="I72" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J72" s="67" t="s">
+      <c r="I72" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J72" s="69" t="s">
         <v>407</v>
       </c>
-      <c r="K72" s="68" t="s">
+      <c r="K72" s="70" t="s">
         <v>450</v>
       </c>
       <c r="L72" s="55">
@@ -5223,75 +5218,75 @@
         <v>14.82</v>
       </c>
     </row>
-    <row r="73" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A73" s="14"/>
       <c r="B73" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B73) - ROW($B$9)</f>
         <v>64</v>
       </c>
       <c r="C73" s="51">
         <v>1</v>
       </c>
-      <c r="D73" s="66" t="s">
+      <c r="D73" s="68" t="s">
         <v>104</v>
       </c>
-      <c r="E73" s="66" t="s">
+      <c r="E73" s="68" t="s">
         <v>171</v>
       </c>
-      <c r="F73" s="66" t="s">
+      <c r="F73" s="68" t="s">
         <v>238</v>
       </c>
-      <c r="G73" s="66" t="s">
+      <c r="G73" s="68" t="s">
         <v>271</v>
       </c>
-      <c r="H73" s="66" t="s">
+      <c r="H73" s="68" t="s">
         <v>337</v>
       </c>
-      <c r="I73" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J73" s="66" t="s">
+      <c r="I73" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J73" s="68" t="s">
         <v>408</v>
       </c>
-      <c r="K73" s="69" t="s">
+      <c r="K73" s="71" t="s">
         <v>440</v>
       </c>
       <c r="L73" s="57">
-        <f t="shared" ref="L73" si="33">C73*K73</f>
+        <f t="shared" ref="L73" si="31">C73*K73</f>
         <v>0.45</v>
       </c>
     </row>
     <row r="74" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A74" s="14"/>
       <c r="B74" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B74) - ROW($B$9)</f>
         <v>65</v>
       </c>
       <c r="C74" s="50">
         <v>1</v>
       </c>
-      <c r="D74" s="65" t="s">
+      <c r="D74" s="67" t="s">
         <v>105</v>
       </c>
-      <c r="E74" s="65" t="s">
+      <c r="E74" s="67" t="s">
         <v>170</v>
       </c>
-      <c r="F74" s="67" t="s">
+      <c r="F74" s="69" t="s">
         <v>239</v>
       </c>
-      <c r="G74" s="67" t="s">
+      <c r="G74" s="69" t="s">
         <v>271</v>
       </c>
-      <c r="H74" s="67" t="s">
+      <c r="H74" s="69" t="s">
         <v>338</v>
       </c>
-      <c r="I74" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J74" s="67" t="s">
+      <c r="I74" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J74" s="69" t="s">
         <v>409</v>
       </c>
-      <c r="K74" s="68" t="s">
+      <c r="K74" s="70" t="s">
         <v>451</v>
       </c>
       <c r="L74" s="55">
@@ -5299,75 +5294,75 @@
         <v>0.66</v>
       </c>
     </row>
-    <row r="75" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A75" s="14"/>
       <c r="B75" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B75) - ROW($B$9)</f>
         <v>66</v>
       </c>
       <c r="C75" s="51">
         <v>1</v>
       </c>
-      <c r="D75" s="66" t="s">
+      <c r="D75" s="68" t="s">
         <v>106</v>
       </c>
-      <c r="E75" s="66" t="s">
+      <c r="E75" s="68" t="s">
         <v>172</v>
       </c>
-      <c r="F75" s="66" t="s">
+      <c r="F75" s="68" t="s">
         <v>240</v>
       </c>
-      <c r="G75" s="66" t="s">
+      <c r="G75" s="68" t="s">
         <v>271</v>
       </c>
-      <c r="H75" s="66" t="s">
+      <c r="H75" s="68" t="s">
         <v>339</v>
       </c>
-      <c r="I75" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J75" s="66" t="s">
+      <c r="I75" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J75" s="68" t="s">
         <v>410</v>
       </c>
-      <c r="K75" s="69" t="s">
+      <c r="K75" s="71" t="s">
         <v>452</v>
       </c>
       <c r="L75" s="57">
-        <f t="shared" ref="L75" si="34">C75*K75</f>
+        <f t="shared" ref="L75" si="32">C75*K75</f>
         <v>6.42</v>
       </c>
     </row>
     <row r="76" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A76" s="14"/>
       <c r="B76" s="48">
-        <f t="shared" si="17"/>
+        <f>ROW(B76) - ROW($B$9)</f>
         <v>67</v>
       </c>
       <c r="C76" s="50">
         <v>1</v>
       </c>
-      <c r="D76" s="65" t="s">
+      <c r="D76" s="67" t="s">
         <v>107</v>
       </c>
-      <c r="E76" s="65" t="s">
+      <c r="E76" s="67" t="s">
         <v>173</v>
       </c>
-      <c r="F76" s="67" t="s">
+      <c r="F76" s="69" t="s">
         <v>241</v>
       </c>
-      <c r="G76" s="67" t="s">
+      <c r="G76" s="69" t="s">
         <v>272</v>
       </c>
-      <c r="H76" s="67" t="s">
+      <c r="H76" s="69" t="s">
         <v>340</v>
       </c>
-      <c r="I76" s="67" t="s">
-        <v>343</v>
-      </c>
-      <c r="J76" s="67" t="s">
+      <c r="I76" s="69" t="s">
+        <v>343</v>
+      </c>
+      <c r="J76" s="69" t="s">
         <v>411</v>
       </c>
-      <c r="K76" s="68" t="s">
+      <c r="K76" s="70" t="s">
         <v>453</v>
       </c>
       <c r="L76" s="55">
@@ -5375,51 +5370,51 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="77" spans="1:12" s="3" customFormat="1" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:12" s="3" customFormat="1" ht="13.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A77" s="14"/>
       <c r="B77" s="49">
-        <f t="shared" si="17"/>
+        <f>ROW(B77) - ROW($B$9)</f>
         <v>68</v>
       </c>
       <c r="C77" s="51">
         <v>1</v>
       </c>
-      <c r="D77" s="66" t="s">
+      <c r="D77" s="68" t="s">
         <v>108</v>
       </c>
-      <c r="E77" s="66" t="s">
+      <c r="E77" s="68" t="s">
         <v>172</v>
       </c>
-      <c r="F77" s="66" t="s">
+      <c r="F77" s="68" t="s">
         <v>242</v>
       </c>
-      <c r="G77" s="66" t="s">
+      <c r="G77" s="68" t="s">
         <v>271</v>
       </c>
-      <c r="H77" s="66" t="s">
+      <c r="H77" s="68" t="s">
         <v>341</v>
       </c>
-      <c r="I77" s="66" t="s">
-        <v>343</v>
-      </c>
-      <c r="J77" s="66" t="s">
+      <c r="I77" s="68" t="s">
+        <v>343</v>
+      </c>
+      <c r="J77" s="68" t="s">
         <v>412</v>
       </c>
-      <c r="K77" s="69" t="s">
+      <c r="K77" s="71" t="s">
         <v>454</v>
       </c>
       <c r="L77" s="57">
-        <f t="shared" ref="L77" si="35">C77*K77</f>
+        <f t="shared" ref="L77" si="33">C77*K77</f>
         <v>4.41</v>
       </c>
     </row>
     <row r="78" spans="1:12" x14ac:dyDescent="0.2">
       <c r="A78" s="14"/>
-      <c r="B78" s="73" t="s">
+      <c r="B78" s="58" t="s">
         <v>19</v>
       </c>
-      <c r="C78" s="74"/>
-      <c r="D78" s="74"/>
+      <c r="C78" s="59"/>
+      <c r="D78" s="59"/>
       <c r="E78" s="47"/>
       <c r="F78" s="46"/>
       <c r="G78" s="7" t="s">
@@ -5535,7 +5530,7 @@
       <c r="A1" s="43" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="70" t="s">
+      <c r="B1" s="72" t="s">
         <v>455</v>
       </c>
     </row>
@@ -5543,7 +5538,7 @@
       <c r="A2" s="42" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="71" t="s">
+      <c r="B2" s="73" t="s">
         <v>31</v>
       </c>
     </row>
@@ -5551,7 +5546,7 @@
       <c r="A3" s="43" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="72" t="s">
+      <c r="B3" s="74" t="s">
         <v>32</v>
       </c>
     </row>
@@ -5559,7 +5554,7 @@
       <c r="A4" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="B4" s="71" t="s">
+      <c r="B4" s="73" t="s">
         <v>31</v>
       </c>
     </row>
@@ -5567,7 +5562,7 @@
       <c r="A5" s="43" t="s">
         <v>4</v>
       </c>
-      <c r="B5" s="72" t="s">
+      <c r="B5" s="74" t="s">
         <v>455</v>
       </c>
     </row>
@@ -5575,7 +5570,7 @@
       <c r="A6" s="42" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="71" t="s">
+      <c r="B6" s="73" t="s">
         <v>35</v>
       </c>
     </row>
@@ -5583,7 +5578,7 @@
       <c r="A7" s="43" t="s">
         <v>6</v>
       </c>
-      <c r="B7" s="72" t="s">
+      <c r="B7" s="74" t="s">
         <v>456</v>
       </c>
     </row>
@@ -5591,7 +5586,7 @@
       <c r="A8" s="42" t="s">
         <v>7</v>
       </c>
-      <c r="B8" s="71" t="s">
+      <c r="B8" s="73" t="s">
         <v>34</v>
       </c>
     </row>
@@ -5599,7 +5594,7 @@
       <c r="A9" s="43" t="s">
         <v>8</v>
       </c>
-      <c r="B9" s="72" t="s">
+      <c r="B9" s="74" t="s">
         <v>33</v>
       </c>
     </row>
@@ -5607,7 +5602,7 @@
       <c r="A10" s="42" t="s">
         <v>9</v>
       </c>
-      <c r="B10" s="71" t="s">
+      <c r="B10" s="73" t="s">
         <v>457</v>
       </c>
     </row>
@@ -5615,7 +5610,7 @@
       <c r="A11" s="43" t="s">
         <v>10</v>
       </c>
-      <c r="B11" s="72" t="s">
+      <c r="B11" s="74" t="s">
         <v>458</v>
       </c>
     </row>
@@ -5623,7 +5618,7 @@
       <c r="A12" s="42" t="s">
         <v>11</v>
       </c>
-      <c r="B12" s="71" t="s">
+      <c r="B12" s="73" t="s">
         <v>458</v>
       </c>
     </row>
@@ -5631,7 +5626,7 @@
       <c r="A13" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="B13" s="72" t="s">
+      <c r="B13" s="74" t="s">
         <v>459</v>
       </c>
     </row>
@@ -5639,7 +5634,7 @@
       <c r="A14" s="42" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="71" t="s">
+      <c r="B14" s="73" t="s">
         <v>460</v>
       </c>
     </row>
@@ -5647,7 +5642,7 @@
       <c r="A15" s="43" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="72" t="s">
+      <c r="B15" s="74" t="s">
         <v>461</v>
       </c>
     </row>
@@ -5655,7 +5650,7 @@
       <c r="A16" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="B16" s="71" t="s">
+      <c r="B16" s="73" t="s">
         <v>462</v>
       </c>
     </row>

</xml_diff>